<commit_message>
Los 18 cursos en formato nuevo (UX3): un libro por lección, mosaicos con submosaicos y práctica incrustada
- Your Money, Tu Patrimonio, Tu Talento, Tu Turno, Tu Trabajo, Tu Idea, Tu Negocio MX y EE. UU., Your Business: nombres amables por parte y regeneración completa.
- Instructivo en inglés adaptado al formato nuevo (también corrige Back Home).
- Vista previa local de cursos en inglés, toda en inglés.
- Libro opcional en inglés: «Further reading».

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P5F6YBSbmgYFHyY7RUeBgK
</commit_message>
<xml_diff>
--- a/cursos/tu_negocio_mx/moodle/herramientas/Herramientas_TNDF.xlsx
+++ b/cursos/tu_negocio_mx/moodle/herramientas/Herramientas_TNDF.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Precio" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Equilibrio" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Flujo" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Adelantos" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1526,4 +1527,205 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Adelantos a mi equipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Escribe solo en las celdas rosas. Usa montos inventados o aproximados; este archivo es tuyo y no se comparte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Persona (apodo)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Adelanto</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Descuento por pago</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Pagos hechos</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Falta</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Pagos que faltan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="n"/>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="10" t="n"/>
+      <c r="E5" s="8">
+        <f>MAX(B5-C5*D5,0)</f>
+        <v/>
+      </c>
+      <c r="F5" s="11">
+        <f>IF(C5&gt;0,ROUNDUP(E5/C5,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="n"/>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="10" t="n"/>
+      <c r="E6" s="8">
+        <f>MAX(B6-C6*D6,0)</f>
+        <v/>
+      </c>
+      <c r="F6" s="11">
+        <f>IF(C6&gt;0,ROUNDUP(E6/C6,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="n"/>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="10" t="n"/>
+      <c r="E7" s="8">
+        <f>MAX(B7-C7*D7,0)</f>
+        <v/>
+      </c>
+      <c r="F7" s="11">
+        <f>IF(C7&gt;0,ROUNDUP(E7/C7,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="n"/>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="10" t="n"/>
+      <c r="E8" s="8">
+        <f>MAX(B8-C8*D8,0)</f>
+        <v/>
+      </c>
+      <c r="F8" s="11">
+        <f>IF(C8&gt;0,ROUNDUP(E8/C8,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="n"/>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="10" t="n"/>
+      <c r="E9" s="8">
+        <f>MAX(B9-C9*D9,0)</f>
+        <v/>
+      </c>
+      <c r="F9" s="11">
+        <f>IF(C9&gt;0,ROUNDUP(E9/C9,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="n"/>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="8">
+        <f>MAX(B10-C10*D10,0)</f>
+        <v/>
+      </c>
+      <c r="F10" s="11">
+        <f>IF(C10&gt;0,ROUNDUP(E10/C10,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="n"/>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="8">
+        <f>MAX(B11-C11*D11,0)</f>
+        <v/>
+      </c>
+      <c r="F11" s="11">
+        <f>IF(C11&gt;0,ROUNDUP(E11/C11,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="n"/>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="8">
+        <f>MAX(B12-C12*D12,0)</f>
+        <v/>
+      </c>
+      <c r="F12" s="11">
+        <f>IF(C12&gt;0,ROUNDUP(E12/C12,0),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Fondo de adelantos del mes</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Me queda en el fondo</t>
+        </is>
+      </c>
+      <c r="B15" s="8">
+        <f>B14-SUM(B5:B12)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>